<commit_message>
Make workbook tasks clearer: numbered task boxes, cell hints, and better legends
</commit_message>
<xml_diff>
--- a/workbooks/unit-a-foundations.xlsx
+++ b/workbooks/unit-a-foundations.xlsx
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,7 +52,7 @@
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00777777"/>
+      <color rgb="00555555"/>
       <sz val="9"/>
     </font>
     <font>
@@ -62,13 +62,37 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B45309"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F4E8C"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <i val="1"/>
+      <color rgb="001F4E8C"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Courier New"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00777777"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -85,8 +109,18 @@
         <fgColor rgb="001F2937"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCEEFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F8FF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -94,11 +128,69 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="004F9DFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="004F9DFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="004F9DFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="004F9DFF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="004F9DFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="004F9DFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="004F9DFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="004F9DFF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="004F9DFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="004F9DFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="004F9DFF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="004F9DFF"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="004F9DFF"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="004F9DFF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -107,9 +199,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -184,6 +292,72 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Excel for Finance course</author>
+  </authors>
+  <commentList>
+    <comment ref="B9" authorId="0" shapeId="0">
+      <text>
+        <t>Type a formula here that grows B8 by the rate in B5.
+Lock B5 with $ so it still works when copied down.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Excel for Finance course</author>
+  </authors>
+  <commentList>
+    <comment ref="B10" authorId="0" shapeId="0">
+      <text>
+        <t>Type =SUM(B6:B8) here.</t>
+      </text>
+    </comment>
+    <comment ref="B11" authorId="0" shapeId="0">
+      <text>
+        <t>Type =AVERAGE(B6:B8) here.</t>
+      </text>
+    </comment>
+    <comment ref="B12" authorId="0" shapeId="0">
+      <text>
+        <t>Type =MAX(B6:B8) here.</t>
+      </text>
+    </comment>
+    <comment ref="B13" authorId="0" shapeId="0">
+      <text>
+        <t>Type =MIN(B6:B8) here.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Excel for Finance course</author>
+  </authors>
+  <commentList>
+    <comment ref="D6" authorId="0" shapeId="0">
+      <text>
+        <t>Type =IF(B6&gt;C6,"Over","OK") here, then copy down through D9.</t>
+      </text>
+    </comment>
+    <comment ref="E6" authorId="0" shapeId="0">
+      <text>
+        <t>Type =IFERROR(B6/C6-1,"n/a") here, then copy down through E9.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -475,7 +649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -506,53 +680,60 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Each tab below matches a module from the website. Read the task at the top of the tab, then type your formula into the yellow cell(s).</t>
+          <t>Each tab has a blue 'YOUR TASK' box with numbered steps — read it first.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Compare your work against the 'Answer Key' tab at the end — it recalculates live from whichever sheet you're on.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+          <t>Yellow cells also have a small red comment triangle in the corner — hover over one for a quick reminder of exactly what to type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Compare your work against the 'Answer Key' tab at the end — it recalculates live from whichever sheet you're on, so it updates as you fill things in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Color legend:</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Yellow fill</t>
         </is>
       </c>
-      <c r="B9">
+      <c r="B10">
         <f> a cell you should fill in</f>
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Blue text</t>
         </is>
       </c>
-      <c r="B10">
+      <c r="B11">
         <f> a hardcoded input/assumption</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Black text</t>
         </is>
       </c>
-      <c r="B11">
+      <c r="B12">
         <f> a formula</f>
         <v/>
       </c>
@@ -568,7 +749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -592,7 +773,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Yellow cells are for you to fill in. Everything else is provided.</t>
+          <t>🟡 Yellow cell = type something here.   🔵 Blue text = a given input.   Black text = a formula already provided.</t>
         </is>
       </c>
     </row>
@@ -607,14 +788,20 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="6"/>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Fill in the yellow cells below ↓</t>
+        </is>
+      </c>
+    </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
@@ -656,21 +843,66 @@
     </row>
     <row r="12"/>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Task: in B9, write a formula that grows B8 by the rate in B5. Use an absolute reference for B5 so the formula still works when copied down to B10 and B11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>✏️  YOUR TASK</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="12" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>1. In cell B9, write a formula that grows B8 by the growth rate in B5.</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="n"/>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>2. Use an absolute reference for B5 (like $B$5) so the SAME formula still works when you copy it down to B10 and B11.</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>3. Copy B9 down through B11 (select B9, drag its fill handle down, or copy/paste).</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>💡 If B10 and B11 come out as 0 or blank, you probably copied a formula that used a relative (unlocked) reference to B5.</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="16" t="n"/>
+      <c r="F17" s="17" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="8">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A13:F14"/>
+    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -680,7 +912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -704,18 +936,18 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Yellow cells are for you to fill in. Everything else is provided.</t>
+          <t>🟡 Yellow cell = type something here.   🔵 Blue text = a given input.   Black text = a formula already provided.</t>
         </is>
       </c>
     </row>
     <row r="4"/>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Revenue ($000)</t>
         </is>
@@ -786,21 +1018,66 @@
     </row>
     <row r="14"/>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Task: fill B10:B13 with SUM, AVERAGE, MAX, and MIN of B6:B8.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16"/>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>✏️  YOUR TASK</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="12" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>1. In B10, write =SUM(B6:B8) to total the three months of revenue.</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>2. In B11, write =AVERAGE(B6:B8).</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>3. In B12, write =MAX(B6:B8) — the single best month.</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>4. In B13, write =MIN(B6:B8) — the single worst month.</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="n"/>
+      <c r="C19" s="16" t="n"/>
+      <c r="D19" s="16" t="n"/>
+      <c r="E19" s="16" t="n"/>
+      <c r="F19" s="17" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="8">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A15:F16"/>
+    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -810,7 +1087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -837,32 +1114,32 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Yellow cells are for you to fill in. Everything else is provided.</t>
+          <t>🟡 Yellow cell = type something here.   🔵 Blue text = a given input.   Black text = a formula already provided.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>Variance %</t>
         </is>
@@ -929,22 +1206,57 @@
       <c r="E9" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Task: in D6:D9 write =IF(actual&gt;budget,"Over","OK"). In E6:E9 write =IFERROR(actual/budget-1,"n/a") — row 8 has a zero budget, which is exactly why IFERROR matters.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
-    <row r="13"/>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>✏️  YOUR TASK</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="12" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>1. In D6, write =IF(B6&gt;C6,"Over","OK") — then copy it down through D9.</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>2. In E6, write =IFERROR(B6/C6-1,"n/a") — then copy it down through E9.</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="n"/>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>3. Look at row 8 (R&amp;D): its budget is $0. Without IFERROR that formula would show #DIV/0! — with it, you get "n/a" instead.</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="n"/>
+      <c r="C14" s="16" t="n"/>
+      <c r="D14" s="16" t="n"/>
+      <c r="E14" s="16" t="n"/>
+      <c r="F14" s="17" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="7">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A11:F13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -971,22 +1283,22 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Module</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>Cell</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>Correct formula</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>Live check</t>
         </is>
@@ -1003,7 +1315,7 @@
           <t>B9</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>ƒ =B8*(1+$B$5)</t>
         </is>
@@ -1024,7 +1336,7 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>ƒ =B9*(1+$B$5)</t>
         </is>
@@ -1045,7 +1357,7 @@
           <t>B11</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="19" t="inlineStr">
         <is>
           <t>ƒ =B10*(1+$B$5)</t>
         </is>
@@ -1066,7 +1378,7 @@
           <t>B10 (Total)</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>ƒ =SUM(B6:B8)</t>
         </is>
@@ -1087,7 +1399,7 @@
           <t>B11 (Average)</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="19" t="inlineStr">
         <is>
           <t>ƒ =AVERAGE(B6:B8)</t>
         </is>
@@ -1108,7 +1420,7 @@
           <t>B12 (Highest)</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>ƒ =MAX(B6:B8)</t>
         </is>
@@ -1129,7 +1441,7 @@
           <t>B13 (Lowest)</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="19" t="inlineStr">
         <is>
           <t>ƒ =MIN(B6:B8)</t>
         </is>
@@ -1150,7 +1462,7 @@
           <t>D6:D9</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="19" t="inlineStr">
         <is>
           <t>ƒ =IF(B6&gt;C6,"Over","OK")</t>
         </is>
@@ -1171,7 +1483,7 @@
           <t>E6:E9</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C12" s="19" t="inlineStr">
         <is>
           <t>ƒ =IFERROR(B6/C6-1,"n/a")</t>
         </is>
@@ -1182,7 +1494,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>Note: 'Live check' pulls today's value from your own sheet, so once you fill in the yellow cells correctly it will match what you typed.</t>
         </is>

</xml_diff>